<commit_message>
feat: task_list_sejoong에 분析대상 컬럼 추가
공휴일전표·중복전표=전체, 벤포드분析·거액전표·상세검색·라운드넘버=당기

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal_analyzer/sejoong/task_list_sejoong.xlsx
+++ b/journal_analyzer/sejoong/task_list_sejoong.xlsx
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -581,6 +581,11 @@
           <t>실행여부</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>분析대상</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -601,6 +606,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -621,6 +631,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -641,6 +656,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -661,6 +681,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -681,6 +706,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -699,6 +729,11 @@
       <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>당기</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: task_list_sejoong에 특수관계자 분析 추가
- 분析목록 11번(특수관계자분析, 전체) 추가
- 특수관계자 파라미터 시트 생성 (거래처명/실행여부 컬럼)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal_analyzer/sejoong/task_list_sejoong.xlsx
+++ b/journal_analyzer/sejoong/task_list_sejoong.xlsx
@@ -13,6 +13,7 @@
     <sheet name="거액전표" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="상세검색" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="라운드넘버" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="특수관계자" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -734,6 +735,31 @@
       <c r="E7" t="inlineStr">
         <is>
           <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>특수관계자분析</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>특수관계자 거래처 거래 추출 → 특수관계자 시트 참조</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>전체</t>
         </is>
       </c>
     </row>
@@ -1326,4 +1352,51 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>거래처명</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: task_list_sejoong 분析목록을 원본 analysis.py 메뉴(1~19번) 기준으로 전면 재정비
- 원본 메뉴명으로 분析명 통일 (거래처 전기/당기 비교, 벤포드 분析 등)
- 전체 18개 분析항목 등록 (실행Y: 2,3,10,11 / 나머지 N)
- 분析번호가 main_analyzer ANALYSIS_REGISTRY와 정확히 일치

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal_analyzer/sejoong/task_list_sejoong.xlsx
+++ b/journal_analyzer/sejoong/task_list_sejoong.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,25 +15,35 @@
     <sheet name="특수관계자" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <sz val="8"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -46,17 +55,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
+        <fgColor rgb="FF2F5496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCE6F1"/>
+        <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,23 +79,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -97,9 +107,15 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -463,7 +479,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -495,10 +511,10 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>㈜그래피</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
+          <t>㈜세중</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -506,10 +522,8 @@
           <t>StartDate</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2025-01-01</t>
-        </is>
+      <c r="B3" s="4" t="n">
+        <v>46023</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
@@ -523,12 +537,10 @@
           <t>EndDate</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>2025-12-31</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="B4" s="5" t="n">
+        <v>46387</v>
+      </c>
+      <c r="C4" s="2" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -537,9 +549,9 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C5" s="3" t="inlineStr"/>
+        <v>2026</v>
+      </c>
+      <c r="C5" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -552,8 +564,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -590,16 +602,16 @@
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>공휴일전표</t>
+          <t>거래처 전기/당기 비교</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>토·일·공휴일 입력 전표 추출 (파라미터 불필요)</t>
+          <t>전기/당기 거래처별 금액 비교 → 거래처비교 시트 참조</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -615,16 +627,16 @@
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>중복전표</t>
+          <t>벤포드 분析</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>날짜·계정·금액·거래처 중복 전표 추출 (파라미터 불필요)</t>
+          <t>첫째자리 빈도 벤포드 기댓값 비교 → 벤포드분析 시트 참조</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -634,27 +646,27 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>당기</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>벤포드분析</t>
+          <t>데이터 개요</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>첫째자리 빈도 벤포드 기댓값 비교 → 벤포드분析 시트 참조</t>
+          <t>전체 데이터 건수/금액 요약 (파라미터 불필요)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -669,17 +681,17 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>거액전표</t>
+          <t>계정명 리스트</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>상위 N% 거액 전표 추출 → 거액전표 시트 참조</t>
+          <t>계정명 목록 및 금액 통계 (파라미터 불필요)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -694,17 +706,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>상세검색</t>
+          <t>사원별 집계</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>계정/거래처/적요 복합 조건 검색 → 상세검색 시트 참조</t>
+          <t>사원별 차변/대변 계정 집계 (파라미터 불필요)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -715,21 +727,21 @@
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>라운드넘버</t>
+          <t>일자차이 분析</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>특정 배수 단위 금액 탐지 → 라운드넘버 시트 참조</t>
+          <t>전표일자 vs 등록일자 N일 이상 지연 전표 → 일자차이분析 시트 참조</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -740,24 +752,299 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>상대계정 분析</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>특정 계정의 상대계정 분析 → 상대계정분析 시트 참조</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>키워드 검색</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>적요 키워드 검색 → 키워드검색 시트 참조</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>라운드넘버 분析</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>특정 배수 단위 금액 탐지 → 라운드넘버 시트 참조</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>11</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>특수관계자분析</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>특수관계자 분析</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>특수관계자 거래처 거래 추출 → 특수관계자 시트 참조</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>자산 vs 부채 교차</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>자산/부채 동시 발생 거래처 分析</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>매출 vs 비용 교차</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>매출/비용 동시 발생 거래처 分析</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>심층분析 (계정별 Top)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>계정별 거래처 Top N 추출 → 심층분析 시트 참조</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>AI 계정별 분析</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>계정별 월별 추이 및 샘플 추출 → AI계정별분析 시트 참조</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>데이터·헤더 확인</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>컬럼 인식 현황 점검 (파라미터 불필요)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>거래처 분析</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>특정 거래처 복합조건 상세 分析 → 거래처분析 시트 참조</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>벤포드 이탈 상세 추출</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>벤포드 이탈 전표 상세 추출 → 벤포드이탈 시트 참조</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>월별 전계정 分析</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>전 계정 월별 차변/대변 집계 (파라미터 불필요)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
@@ -775,7 +1062,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -821,7 +1108,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -839,7 +1126,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -857,7 +1144,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -875,7 +1162,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -911,7 +1198,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1034,15 +1321,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1104,7 +1390,7 @@
           <t>GRAPHY SMA</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>대변만</t>
@@ -1134,7 +1420,7 @@
           <t>GRAPHY SMA</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>차변만</t>
@@ -1159,8 +1445,8 @@
           <t>기계장치</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>차변만</t>
@@ -1187,8 +1473,8 @@
           <t>보통예금</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>양방향</t>
@@ -1210,8 +1496,8 @@
           <t>특정적요_검색</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
           <t>가지급</t>
@@ -1242,7 +1528,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1322,7 +1608,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1361,13 +1647,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>거래처명</t>
-        </is>
+      <c r="A1" t="n">
+        <v>11</v>
       </c>
       <c r="B1" t="inlineStr">
         <is>

</xml_diff>